<commit_message>
MAERSK: Commercial Invoice No as Order No; multi-FCR invoices
- Order No. = "Commercial Invoice No:" again (joined when the list of
  numbers wraps across lines); MBL NO. back to N/A, per the user's
  updated reference Excel.
- One invoice can cover several FCR shipments: split by "FCR xxx"
  blocks so each row carries its own B/L (FCR), POL/POD, ETD/ETA,
  shipper and volume (the block's M3 quantity).
- Handle "Min. Quantity Price" lines where the charge amount is printed
  on its own line instead of the item line.
- Item table now ends at the block subtotal line instead of
  "Total Packages" (absent on earlier pages of multi-page invoices).
- Add sample3 (5617470598, 10 FCRs / 40 items); reference generated
  from the extraction after every block subtotal and the invoice
  Net value / Amount Due audit matched.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_samples/MAERSK/sample1_ref.xlsx
+++ b/test_samples/MAERSK/sample1_ref.xlsx
@@ -656,7 +656,7 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0903164786</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
@@ -670,8 +670,10 @@
           <t>JKT3320212</t>
         </is>
       </c>
-      <c r="L2" s="0" t="n">
-        <v>5617840405</v>
+      <c r="L2" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
         <is>
@@ -729,7 +731,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0903164786</t>
         </is>
       </c>
       <c r="I3" s="3" t="n">
@@ -743,8 +745,10 @@
           <t>JKT3320212</t>
         </is>
       </c>
-      <c r="L3" s="0" t="n">
-        <v>5617840405</v>
+      <c r="L3" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M3" s="0" t="inlineStr">
         <is>
@@ -802,7 +806,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0903164786</t>
         </is>
       </c>
       <c r="I4" s="3" t="n">
@@ -816,8 +820,10 @@
           <t>JKT3320212</t>
         </is>
       </c>
-      <c r="L4" s="0" t="n">
-        <v>5617840405</v>
+      <c r="L4" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M4" s="0" t="inlineStr">
         <is>
@@ -875,7 +881,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0903164786</t>
         </is>
       </c>
       <c r="I5" s="3" t="n">
@@ -889,8 +895,10 @@
           <t>JKT3320212</t>
         </is>
       </c>
-      <c r="L5" s="0" t="n">
-        <v>5617840405</v>
+      <c r="L5" s="0" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M5" s="0" t="inlineStr">
         <is>
@@ -931,9 +939,6 @@
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="R12" s="1" t="n"/>
     </row>

</xml_diff>